<commit_message>
Update content calendar - Topic 4
</commit_message>
<xml_diff>
--- a/carousel-data/content-calendar.xlsx
+++ b/carousel-data/content-calendar.xlsx
@@ -4584,7 +4584,32 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>trust-killers, build-trust, remote-rituals</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>7, 8, 8</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>LinkedIn, LinkedIn Page, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>3 carousels: trust killers, building trust principles, remote rituals</t>
         </is>
       </c>
     </row>

</xml_diff>